<commit_message>
last update at 12pm saturday after complete all reports and ordering
</commit_message>
<xml_diff>
--- a/july 2026/Daily Reports/LMT Orders.xlsx
+++ b/july 2026/Daily Reports/LMT Orders.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\786\Desktop\Elite-Git\july 2026\Daily Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC201AFF-1F68-46CC-BF4C-64F961CC658F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8784412-C76C-43D4-96D5-277BD21D0013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -547,25 +547,25 @@
     <t xml:space="preserve">Rainbow Behria Town </t>
   </si>
   <si>
-    <t xml:space="preserve">Raja Sab </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Askari </t>
-  </si>
-  <si>
     <t xml:space="preserve">Swera Punjab Society </t>
   </si>
   <si>
-    <t>Euro NFC</t>
-  </si>
-  <si>
     <t>18/07/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Rubaika </t>
-  </si>
-  <si>
     <t xml:space="preserve">Jalal Sons Johar Town </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Askari  Punjab Society </t>
+  </si>
+  <si>
+    <t>Rubaika Velencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Euro NFC </t>
+  </si>
+  <si>
+    <t>Raja Sab Wapda Town</t>
   </si>
 </sst>
 </file>
@@ -1473,7 +1473,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="191">
+  <cellXfs count="190">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1871,6 +1871,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1907,45 +1946,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1968,9 +1968,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2508,14 +2505,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="157">
+      <c r="B1" s="170">
         <f ca="1">TODAY()</f>
         <v>46221</v>
       </c>
-      <c r="C1" s="157"/>
-      <c r="D1" s="157"/>
-      <c r="E1" s="157"/>
-      <c r="F1" s="157"/>
+      <c r="C1" s="170"/>
+      <c r="D1" s="170"/>
+      <c r="E1" s="170"/>
+      <c r="F1" s="170"/>
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
       <c r="I1" s="10"/>
@@ -2537,10 +2534,10 @@
       <c r="Y1" s="10"/>
     </row>
     <row r="2" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="179" t="s">
+      <c r="A2" s="167" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="158" t="s">
+      <c r="B2" s="171" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="12" t="s">
@@ -2573,13 +2570,13 @@
       <c r="L2" s="15">
         <v>120</v>
       </c>
-      <c r="M2" s="171"/>
-      <c r="N2" s="172"/>
-      <c r="O2" s="173"/>
-      <c r="P2" s="174" t="s">
+      <c r="M2" s="159"/>
+      <c r="N2" s="160"/>
+      <c r="O2" s="161"/>
+      <c r="P2" s="162" t="s">
         <v>14</v>
       </c>
-      <c r="Q2" s="175"/>
+      <c r="Q2" s="163"/>
       <c r="R2" s="18">
         <v>0.05</v>
       </c>
@@ -2598,8 +2595,8 @@
       <c r="Y2" s="20"/>
     </row>
     <row r="3" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="179"/>
-      <c r="B3" s="159"/>
+      <c r="A3" s="167"/>
+      <c r="B3" s="172"/>
       <c r="C3" s="23" t="s">
         <v>15</v>
       </c>
@@ -2630,29 +2627,29 @@
       <c r="L3" s="29">
         <v>72.64</v>
       </c>
-      <c r="M3" s="176" t="s">
+      <c r="M3" s="164" t="s">
         <v>11</v>
       </c>
-      <c r="N3" s="177"/>
-      <c r="O3" s="178"/>
+      <c r="N3" s="165"/>
+      <c r="O3" s="166"/>
       <c r="P3" s="71"/>
       <c r="Q3" s="72"/>
-      <c r="R3" s="161" t="s">
+      <c r="R3" s="174" t="s">
         <v>16</v>
       </c>
-      <c r="S3" s="162"/>
-      <c r="T3" s="162"/>
-      <c r="U3" s="163"/>
-      <c r="V3" s="164" t="s">
+      <c r="S3" s="175"/>
+      <c r="T3" s="175"/>
+      <c r="U3" s="176"/>
+      <c r="V3" s="177" t="s">
         <v>17</v>
       </c>
-      <c r="W3" s="165"/>
-      <c r="X3" s="165"/>
-      <c r="Y3" s="166"/>
+      <c r="W3" s="178"/>
+      <c r="X3" s="178"/>
+      <c r="Y3" s="179"/>
     </row>
     <row r="4" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="179"/>
-      <c r="B4" s="160"/>
+      <c r="A4" s="167"/>
+      <c r="B4" s="173"/>
       <c r="C4" s="30" t="s">
         <v>18</v>
       </c>
@@ -11659,10 +11656,10 @@
     </row>
     <row r="132" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A132" s="78"/>
-      <c r="B132" s="167" t="s">
+      <c r="B132" s="180" t="s">
         <v>11</v>
       </c>
-      <c r="C132" s="168"/>
+      <c r="C132" s="181"/>
       <c r="D132" s="88">
         <f t="shared" ref="D132:L132" si="104">SUM(D6:D60)</f>
         <v>2440</v>
@@ -11926,10 +11923,10 @@
       </c>
     </row>
     <row r="136" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B136" s="180" t="s">
+      <c r="B136" s="168" t="s">
         <v>73</v>
       </c>
-      <c r="C136" s="181"/>
+      <c r="C136" s="169"/>
       <c r="D136" s="87">
         <f>SUM(D134:D135)</f>
         <v>0</v>
@@ -12020,10 +12017,10 @@
       </c>
     </row>
     <row r="137" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B137" s="169" t="s">
+      <c r="B137" s="157" t="s">
         <v>11</v>
       </c>
-      <c r="C137" s="170"/>
+      <c r="C137" s="158"/>
       <c r="D137" s="89">
         <f>SUM(D132,D136)</f>
         <v>2440</v>
@@ -12115,17 +12112,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="R3:U3"/>
+    <mergeCell ref="V3:Y3"/>
+    <mergeCell ref="B132:C132"/>
     <mergeCell ref="B137:C137"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="M3:O3"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B136:C136"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="R3:U3"/>
-    <mergeCell ref="V3:Y3"/>
-    <mergeCell ref="B132:C132"/>
   </mergeCells>
   <conditionalFormatting sqref="C45:C59">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
@@ -13947,12 +13944,12 @@
         <v>166</v>
       </c>
       <c r="I41" s="79" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="J41" s="79">
         <v>4</v>
       </c>
-      <c r="K41" s="190" t="s">
+      <c r="K41" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L41" s="79"/>
@@ -13963,15 +13960,15 @@
     </row>
     <row r="42" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H42" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I42" s="190" t="s">
+        <v>174</v>
+      </c>
+      <c r="I42" s="79" t="s">
         <v>170</v>
       </c>
       <c r="J42" s="79">
         <v>8</v>
       </c>
-      <c r="K42" s="190" t="s">
+      <c r="K42" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L42" s="2"/>
@@ -13982,15 +13979,15 @@
     </row>
     <row r="43" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H43" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I43" s="190" t="s">
+        <v>174</v>
+      </c>
+      <c r="I43" s="79" t="s">
         <v>171</v>
       </c>
       <c r="J43" s="79">
         <v>9</v>
       </c>
-      <c r="K43" s="190" t="s">
+      <c r="K43" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L43" s="2"/>
@@ -14001,15 +13998,15 @@
     </row>
     <row r="44" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H44" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I44" s="190" t="s">
+        <v>174</v>
+      </c>
+      <c r="I44" s="79" t="s">
         <v>172</v>
       </c>
       <c r="J44" s="79">
         <v>5</v>
       </c>
-      <c r="K44" s="190" t="s">
+      <c r="K44" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L44" s="2"/>
@@ -14020,15 +14017,15 @@
     </row>
     <row r="45" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H45" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I45" s="190" t="s">
-        <v>173</v>
+        <v>174</v>
+      </c>
+      <c r="I45" s="79" t="s">
+        <v>179</v>
       </c>
       <c r="J45" s="79">
         <v>5</v>
       </c>
-      <c r="K45" s="190" t="s">
+      <c r="K45" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L45" s="2"/>
@@ -14039,15 +14036,15 @@
     </row>
     <row r="46" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H46" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I46" s="190" t="s">
         <v>174</v>
+      </c>
+      <c r="I46" s="79" t="s">
+        <v>176</v>
       </c>
       <c r="J46" s="79">
         <v>8</v>
       </c>
-      <c r="K46" s="190" t="s">
+      <c r="K46" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L46" s="2"/>
@@ -14058,15 +14055,15 @@
     </row>
     <row r="47" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H47" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="I47" s="79" t="s">
         <v>177</v>
-      </c>
-      <c r="I47" s="190" t="s">
-        <v>178</v>
       </c>
       <c r="J47" s="79">
         <v>8</v>
       </c>
-      <c r="K47" s="190" t="s">
+      <c r="K47" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L47" s="2"/>
@@ -14077,15 +14074,15 @@
     </row>
     <row r="48" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H48" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I48" s="190" t="s">
-        <v>175</v>
+        <v>174</v>
+      </c>
+      <c r="I48" s="79" t="s">
+        <v>173</v>
       </c>
       <c r="J48" s="79">
         <v>20</v>
       </c>
-      <c r="K48" s="190" t="s">
+      <c r="K48" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L48" s="2"/>
@@ -14096,15 +14093,15 @@
     </row>
     <row r="49" spans="8:13" x14ac:dyDescent="0.35">
       <c r="H49" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I49" s="190" t="s">
-        <v>176</v>
+        <v>174</v>
+      </c>
+      <c r="I49" s="79" t="s">
+        <v>178</v>
       </c>
       <c r="J49" s="79">
         <v>4</v>
       </c>
-      <c r="K49" s="190" t="s">
+      <c r="K49" s="79" t="s">
         <v>142</v>
       </c>
       <c r="L49" s="2"/>
@@ -14114,7 +14111,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="H1:M40" xr:uid="{A43751F5-4C5F-4082-9A98-9CA12EDC5193}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>

</xml_diff>

<commit_message>
udpated after Stt completed at 18-07
</commit_message>
<xml_diff>
--- a/july 2026/Daily Reports/LMT Orders.xlsx
+++ b/july 2026/Daily Reports/LMT Orders.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\786\Desktop\Elite-Git\july 2026\Daily Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AEB8157-9FA7-4D23-9C9F-A8D2AD41DA6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B002CF2-3AB2-48EF-91A6-4B606911BCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1497,7 +1497,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="199">
+  <cellXfs count="198">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1899,108 +1899,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2010,6 +1908,105 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2546,14 +2543,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="159">
+      <c r="B1" s="165">
         <f ca="1">TODAY()</f>
         <v>46223</v>
       </c>
-      <c r="C1" s="159"/>
-      <c r="D1" s="159"/>
-      <c r="E1" s="159"/>
-      <c r="F1" s="159"/>
+      <c r="C1" s="165"/>
+      <c r="D1" s="165"/>
+      <c r="E1" s="165"/>
+      <c r="F1" s="165"/>
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
       <c r="I1" s="10"/>
@@ -2575,10 +2572,10 @@
       <c r="Y1" s="10"/>
     </row>
     <row r="2" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="181" t="s">
+      <c r="A2" s="187" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="160" t="s">
+      <c r="B2" s="166" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="12" t="s">
@@ -2611,13 +2608,13 @@
       <c r="L2" s="15">
         <v>120</v>
       </c>
-      <c r="M2" s="173"/>
-      <c r="N2" s="174"/>
-      <c r="O2" s="175"/>
-      <c r="P2" s="176" t="s">
+      <c r="M2" s="179"/>
+      <c r="N2" s="180"/>
+      <c r="O2" s="181"/>
+      <c r="P2" s="182" t="s">
         <v>14</v>
       </c>
-      <c r="Q2" s="177"/>
+      <c r="Q2" s="183"/>
       <c r="R2" s="18">
         <v>0.05</v>
       </c>
@@ -2636,8 +2633,8 @@
       <c r="Y2" s="20"/>
     </row>
     <row r="3" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="181"/>
-      <c r="B3" s="161"/>
+      <c r="A3" s="187"/>
+      <c r="B3" s="167"/>
       <c r="C3" s="23" t="s">
         <v>15</v>
       </c>
@@ -2668,29 +2665,29 @@
       <c r="L3" s="29">
         <v>72.64</v>
       </c>
-      <c r="M3" s="178" t="s">
+      <c r="M3" s="184" t="s">
         <v>11</v>
       </c>
-      <c r="N3" s="179"/>
-      <c r="O3" s="180"/>
+      <c r="N3" s="185"/>
+      <c r="O3" s="186"/>
       <c r="P3" s="71"/>
       <c r="Q3" s="72"/>
-      <c r="R3" s="163" t="s">
+      <c r="R3" s="169" t="s">
         <v>16</v>
       </c>
-      <c r="S3" s="164"/>
-      <c r="T3" s="164"/>
-      <c r="U3" s="165"/>
-      <c r="V3" s="166" t="s">
+      <c r="S3" s="170"/>
+      <c r="T3" s="170"/>
+      <c r="U3" s="171"/>
+      <c r="V3" s="172" t="s">
         <v>17</v>
       </c>
-      <c r="W3" s="167"/>
-      <c r="X3" s="167"/>
-      <c r="Y3" s="168"/>
+      <c r="W3" s="173"/>
+      <c r="X3" s="173"/>
+      <c r="Y3" s="174"/>
     </row>
     <row r="4" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="181"/>
-      <c r="B4" s="162"/>
+      <c r="A4" s="187"/>
+      <c r="B4" s="168"/>
       <c r="C4" s="30" t="s">
         <v>18</v>
       </c>
@@ -6372,24 +6369,24 @@
       <c r="B51" s="47">
         <v>47</v>
       </c>
-      <c r="C51" s="193" t="s">
+      <c r="C51" s="159" t="s">
         <v>175</v>
       </c>
-      <c r="D51" s="194"/>
-      <c r="E51" s="195"/>
-      <c r="F51" s="196"/>
-      <c r="G51" s="197">
+      <c r="D51" s="160"/>
+      <c r="E51" s="161"/>
+      <c r="F51" s="162"/>
+      <c r="G51" s="163">
         <v>40</v>
       </c>
-      <c r="H51" s="195">
+      <c r="H51" s="161">
         <v>40</v>
       </c>
       <c r="I51" s="56"/>
-      <c r="J51" s="197">
+      <c r="J51" s="163">
         <v>40</v>
       </c>
-      <c r="K51" s="195"/>
-      <c r="L51" s="196">
+      <c r="K51" s="161"/>
+      <c r="L51" s="162">
         <v>40</v>
       </c>
       <c r="M51" s="48">
@@ -6434,24 +6431,24 @@
       <c r="B52" s="47">
         <v>48</v>
       </c>
-      <c r="C52" s="193" t="s">
+      <c r="C52" s="159" t="s">
         <v>112</v>
       </c>
-      <c r="D52" s="194"/>
-      <c r="E52" s="195"/>
-      <c r="F52" s="196"/>
-      <c r="G52" s="197">
+      <c r="D52" s="160"/>
+      <c r="E52" s="161"/>
+      <c r="F52" s="162"/>
+      <c r="G52" s="163">
         <v>80</v>
       </c>
-      <c r="H52" s="195">
+      <c r="H52" s="161">
         <v>40</v>
       </c>
       <c r="I52" s="56"/>
-      <c r="J52" s="197">
+      <c r="J52" s="163">
         <v>120</v>
       </c>
-      <c r="K52" s="195"/>
-      <c r="L52" s="196">
+      <c r="K52" s="161"/>
+      <c r="L52" s="162">
         <v>120</v>
       </c>
       <c r="M52" s="48">
@@ -6496,22 +6493,22 @@
       <c r="B53" s="47">
         <v>49</v>
       </c>
-      <c r="C53" s="193" t="s">
+      <c r="C53" s="159" t="s">
         <v>184</v>
       </c>
-      <c r="D53" s="194"/>
-      <c r="E53" s="195"/>
-      <c r="F53" s="196"/>
-      <c r="G53" s="197"/>
-      <c r="H53" s="195">
+      <c r="D53" s="160"/>
+      <c r="E53" s="161"/>
+      <c r="F53" s="162"/>
+      <c r="G53" s="163"/>
+      <c r="H53" s="161">
         <v>40</v>
       </c>
       <c r="I53" s="56"/>
-      <c r="J53" s="197">
+      <c r="J53" s="163">
         <v>80</v>
       </c>
-      <c r="K53" s="195"/>
-      <c r="L53" s="196">
+      <c r="K53" s="161"/>
+      <c r="L53" s="162">
         <v>80</v>
       </c>
       <c r="M53" s="48">
@@ -6556,24 +6553,24 @@
       <c r="B54" s="47">
         <v>50</v>
       </c>
-      <c r="C54" s="193" t="s">
+      <c r="C54" s="159" t="s">
         <v>185</v>
       </c>
-      <c r="D54" s="194"/>
-      <c r="E54" s="195"/>
-      <c r="F54" s="196"/>
-      <c r="G54" s="197">
+      <c r="D54" s="160"/>
+      <c r="E54" s="161"/>
+      <c r="F54" s="162"/>
+      <c r="G54" s="163">
         <v>80</v>
       </c>
-      <c r="H54" s="195">
+      <c r="H54" s="161">
         <v>80</v>
       </c>
       <c r="I54" s="56"/>
-      <c r="J54" s="197">
+      <c r="J54" s="163">
         <v>80</v>
       </c>
-      <c r="K54" s="195"/>
-      <c r="L54" s="196">
+      <c r="K54" s="161"/>
+      <c r="L54" s="162">
         <v>80</v>
       </c>
       <c r="M54" s="48">
@@ -6618,24 +6615,24 @@
       <c r="B55" s="47">
         <v>51</v>
       </c>
-      <c r="C55" s="193" t="s">
+      <c r="C55" s="159" t="s">
         <v>186</v>
       </c>
-      <c r="D55" s="194"/>
-      <c r="E55" s="195"/>
-      <c r="F55" s="196"/>
-      <c r="G55" s="197">
+      <c r="D55" s="160"/>
+      <c r="E55" s="161"/>
+      <c r="F55" s="162"/>
+      <c r="G55" s="163">
         <v>80</v>
       </c>
-      <c r="H55" s="195">
+      <c r="H55" s="161">
         <v>80</v>
       </c>
       <c r="I55" s="56"/>
-      <c r="J55" s="197">
+      <c r="J55" s="163">
         <v>80</v>
       </c>
-      <c r="K55" s="195"/>
-      <c r="L55" s="196">
+      <c r="K55" s="161"/>
+      <c r="L55" s="162">
         <v>80</v>
       </c>
       <c r="M55" s="48">
@@ -6680,24 +6677,24 @@
       <c r="B56" s="47">
         <v>52</v>
       </c>
-      <c r="C56" s="193" t="s">
+      <c r="C56" s="159" t="s">
         <v>187</v>
       </c>
-      <c r="D56" s="194"/>
-      <c r="E56" s="195"/>
-      <c r="F56" s="196"/>
-      <c r="G56" s="197">
+      <c r="D56" s="160"/>
+      <c r="E56" s="161"/>
+      <c r="F56" s="162"/>
+      <c r="G56" s="163">
         <v>200</v>
       </c>
-      <c r="H56" s="195">
+      <c r="H56" s="161">
         <v>200</v>
       </c>
       <c r="I56" s="56"/>
-      <c r="J56" s="197">
+      <c r="J56" s="163">
         <v>200</v>
       </c>
-      <c r="K56" s="195"/>
-      <c r="L56" s="196">
+      <c r="K56" s="161"/>
+      <c r="L56" s="162">
         <v>200</v>
       </c>
       <c r="M56" s="48">
@@ -6742,24 +6739,24 @@
       <c r="B57" s="47">
         <v>53</v>
       </c>
-      <c r="C57" s="193" t="s">
+      <c r="C57" s="159" t="s">
         <v>178</v>
       </c>
-      <c r="D57" s="195"/>
-      <c r="E57" s="195"/>
-      <c r="F57" s="195"/>
-      <c r="G57" s="195">
+      <c r="D57" s="161"/>
+      <c r="E57" s="161"/>
+      <c r="F57" s="161"/>
+      <c r="G57" s="161">
         <v>40</v>
       </c>
-      <c r="H57" s="195">
+      <c r="H57" s="161">
         <v>40</v>
       </c>
-      <c r="I57" s="198"/>
-      <c r="J57" s="195">
+      <c r="I57" s="164"/>
+      <c r="J57" s="161">
         <v>40</v>
       </c>
-      <c r="K57" s="195"/>
-      <c r="L57" s="195">
+      <c r="K57" s="161"/>
+      <c r="L57" s="161">
         <v>40</v>
       </c>
       <c r="M57" s="135">
@@ -11779,10 +11776,10 @@
     </row>
     <row r="132" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A132" s="78"/>
-      <c r="B132" s="169" t="s">
+      <c r="B132" s="175" t="s">
         <v>11</v>
       </c>
-      <c r="C132" s="170"/>
+      <c r="C132" s="176"/>
       <c r="D132" s="88">
         <f t="shared" ref="D132:L132" si="104">SUM(D6:D60)</f>
         <v>2440</v>
@@ -12046,10 +12043,10 @@
       </c>
     </row>
     <row r="136" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B136" s="182" t="s">
+      <c r="B136" s="188" t="s">
         <v>73</v>
       </c>
-      <c r="C136" s="183"/>
+      <c r="C136" s="189"/>
       <c r="D136" s="87">
         <f>SUM(D134:D135)</f>
         <v>0</v>
@@ -12140,10 +12137,10 @@
       </c>
     </row>
     <row r="137" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B137" s="171" t="s">
+      <c r="B137" s="177" t="s">
         <v>11</v>
       </c>
-      <c r="C137" s="172"/>
+      <c r="C137" s="178"/>
       <c r="D137" s="89">
         <f>SUM(D132,D136)</f>
         <v>2440</v>
@@ -12280,24 +12277,24 @@
   <sheetData>
     <row r="2" spans="3:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="3:26" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C3" s="186" t="s">
+      <c r="C3" s="192" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="187"/>
-      <c r="E3" s="187"/>
-      <c r="F3" s="187"/>
-      <c r="G3" s="188"/>
-      <c r="H3" s="190" t="s">
+      <c r="D3" s="193"/>
+      <c r="E3" s="193"/>
+      <c r="F3" s="193"/>
+      <c r="G3" s="194"/>
+      <c r="H3" s="196" t="s">
         <v>65</v>
       </c>
-      <c r="I3" s="191"/>
-      <c r="K3" s="185" t="s">
+      <c r="I3" s="197"/>
+      <c r="K3" s="191" t="s">
         <v>69</v>
       </c>
-      <c r="L3" s="185"/>
-      <c r="M3" s="185"/>
-      <c r="N3" s="185"/>
-      <c r="O3" s="185"/>
+      <c r="L3" s="191"/>
+      <c r="M3" s="191"/>
+      <c r="N3" s="191"/>
+      <c r="O3" s="191"/>
     </row>
     <row r="4" spans="3:26" ht="29.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C4" s="103"/>
@@ -12340,22 +12337,22 @@
         <v>51</v>
       </c>
       <c r="D5" s="92">
-        <v>670</v>
+        <v>705</v>
       </c>
       <c r="E5" s="79">
-        <v>735</v>
+        <v>793</v>
       </c>
       <c r="F5" s="79">
         <v>300</v>
       </c>
       <c r="G5" s="106">
         <f>SUM(D5:F5)</f>
-        <v>1705</v>
+        <v>1798</v>
       </c>
       <c r="H5" s="99"/>
       <c r="I5" s="100">
         <f>G5-H5</f>
-        <v>1705</v>
+        <v>1798</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>1</v>
@@ -12380,11 +12377,11 @@
       </c>
       <c r="D6" s="108">
         <f>D5*40</f>
-        <v>26800</v>
+        <v>28200</v>
       </c>
       <c r="E6" s="109">
         <f>E5*40</f>
-        <v>29400</v>
+        <v>31720</v>
       </c>
       <c r="F6" s="109">
         <f>F5*40</f>
@@ -12392,7 +12389,7 @@
       </c>
       <c r="G6" s="110">
         <f>SUM(D6:F6)</f>
-        <v>68200</v>
+        <v>71920</v>
       </c>
       <c r="H6" s="101">
         <f>H5*40</f>
@@ -12400,7 +12397,7 @@
       </c>
       <c r="I6" s="102">
         <f>G6-H6</f>
-        <v>68200</v>
+        <v>71920</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>2</v>
@@ -12527,11 +12524,11 @@
       </c>
       <c r="D9" s="111">
         <f>D8-D5</f>
-        <v>-670</v>
+        <v>-705</v>
       </c>
       <c r="E9" s="111">
         <f>E8-E5</f>
-        <v>-735</v>
+        <v>-793</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>5</v>
@@ -12615,14 +12612,14 @@
       </c>
     </row>
     <row r="11" spans="3:26" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="C11" s="189" t="s">
+      <c r="C11" s="195" t="s">
         <v>62</v>
       </c>
-      <c r="D11" s="189"/>
-      <c r="F11" s="189" t="s">
+      <c r="D11" s="195"/>
+      <c r="F11" s="195" t="s">
         <v>71</v>
       </c>
-      <c r="G11" s="189"/>
+      <c r="G11" s="195"/>
       <c r="K11" s="1" t="s">
         <v>7</v>
       </c>
@@ -12671,7 +12668,7 @@
       </c>
       <c r="G12" s="95">
         <f>D12+G5</f>
-        <v>5139</v>
+        <v>5232</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>11</v>
@@ -12722,12 +12719,12 @@
       </c>
       <c r="G13" s="95">
         <f>G12*40</f>
-        <v>205560</v>
-      </c>
-      <c r="S13" s="184" t="s">
+        <v>209280</v>
+      </c>
+      <c r="S13" s="190" t="s">
         <v>153</v>
       </c>
-      <c r="T13" s="184"/>
+      <c r="T13" s="190"/>
       <c r="U13" s="147">
         <f>SUM(U8:U12)</f>
         <v>100</v>
@@ -12843,13 +12840,13 @@
       </c>
     </row>
     <row r="20" spans="4:17" ht="24" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="D20" s="185" t="s">
+      <c r="D20" s="191" t="s">
         <v>69</v>
       </c>
-      <c r="E20" s="185"/>
-      <c r="F20" s="185"/>
-      <c r="G20" s="185"/>
-      <c r="H20" s="185"/>
+      <c r="E20" s="191"/>
+      <c r="F20" s="191"/>
+      <c r="G20" s="191"/>
+      <c r="H20" s="191"/>
       <c r="K20" s="1" t="s">
         <v>4</v>
       </c>
@@ -14251,16 +14248,16 @@
       <c r="H50" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="I50" s="192" t="s">
+      <c r="I50" s="130" t="s">
         <v>180</v>
       </c>
-      <c r="J50" s="192">
+      <c r="J50" s="130">
         <v>5</v>
       </c>
-      <c r="K50" s="192" t="s">
+      <c r="K50" s="130" t="s">
         <v>142</v>
       </c>
-      <c r="M50" s="192">
+      <c r="M50" s="130">
         <f t="shared" si="1"/>
         <v>200</v>
       </c>
@@ -14269,16 +14266,16 @@
       <c r="H51" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="I51" s="192" t="s">
+      <c r="I51" s="130" t="s">
         <v>181</v>
       </c>
-      <c r="J51" s="192">
+      <c r="J51" s="130">
         <v>300</v>
       </c>
-      <c r="K51" s="192" t="s">
+      <c r="K51" s="130" t="s">
         <v>142</v>
       </c>
-      <c r="M51" s="192">
+      <c r="M51" s="130">
         <f t="shared" si="1"/>
         <v>12000</v>
       </c>
@@ -14287,16 +14284,16 @@
       <c r="H52" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="I52" s="192" t="s">
+      <c r="I52" s="130" t="s">
         <v>182</v>
       </c>
-      <c r="J52" s="192">
+      <c r="J52" s="130">
         <v>305</v>
       </c>
-      <c r="K52" s="192" t="s">
+      <c r="K52" s="130" t="s">
         <v>142</v>
       </c>
-      <c r="M52" s="192">
+      <c r="M52" s="130">
         <f t="shared" si="1"/>
         <v>12200</v>
       </c>

</xml_diff>